<commit_message>
Website update 2026-06-17 13:00:39
</commit_message>
<xml_diff>
--- a/build/source/lasvillasweb.xlsx
+++ b/build/source/lasvillasweb.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\lasvillasdebayamon\web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34E379C2-B15D-422F-B83E-3A0E3B575D7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76E0939A-3A24-4F5C-8628-743F62F18C2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Homepage" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Ultima actualizacion:</t>
   </si>
@@ -109,15 +109,18 @@
 del Consumidor
 de Puerto Rico</t>
   </si>
+  <si>
+    <t>Como cada semana, también hoy tendremos la reunión informal de los miércoles en el gazebo a las 7:00 p. m. Todos son bienvenidos para conversar y discutir temas relacionados con el condominio.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="[$-540A]dddd\,\ mmmm\ d\,\ yyyy\ /\ hh\.mm"/>
+    <numFmt numFmtId="164" formatCode="[$-540A]dddd\,\ mmmm\ d\,\ yyyy\ /\ hh\.mm"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -162,13 +165,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -184,21 +199,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -215,6 +227,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -240,13 +258,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>57151</xdr:colOff>
-      <xdr:row>2</xdr:row>
+      <xdr:row>4</xdr:row>
       <xdr:rowOff>9524</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>3132395</xdr:colOff>
-      <xdr:row>14</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>95785</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -596,18 +614,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Foglio1"/>
-  <dimension ref="A2:D2"/>
+  <dimension ref="A2:A4"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="45.85546875" style="4" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" style="4" customWidth="1"/>
-    <col min="3" max="3" width="19.5703125" style="4" customWidth="1"/>
-    <col min="4" max="4" width="28.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="4"/>
+    <col min="1" max="1" width="45.85546875" style="3" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="19.5703125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="28.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:1" ht="281.25" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+    <row r="2" spans="1:1" ht="112.5" x14ac:dyDescent="0.3">
+      <c r="A2" s="13" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="281.25" x14ac:dyDescent="0.3">
+      <c r="A4" s="11" t="s">
         <v>4</v>
       </c>
     </row>
@@ -624,7 +647,7 @@
   <dimension ref="A2:A5"/>
   <sheetFormatPr defaultColWidth="39.5703125" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16384" width="39.5703125" style="4"/>
+    <col min="1" max="16384" width="39.5703125" style="3"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
@@ -633,12 +656,12 @@
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="7" t="s">
         <v>2</v>
       </c>
     </row>
@@ -657,9 +680,9 @@
   <dimension ref="A2:A14"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.42578125" style="4" customWidth="1"/>
-    <col min="2" max="2" width="16.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="4"/>
+    <col min="1" max="1" width="30.42578125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
@@ -668,51 +691,51 @@
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="8" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" s="9"/>
+      <c r="A6" s="8"/>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="8" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A9" s="9"/>
+      <c r="A9" s="8"/>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="8" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A12" s="9"/>
+      <c r="A12" s="8"/>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -729,9 +752,9 @@
   <dimension ref="A2:B5"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="4"/>
+    <col min="1" max="1" width="30.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -740,13 +763,13 @@
       </c>
     </row>
     <row r="4" spans="1:2" ht="75" x14ac:dyDescent="0.3">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="5"/>
+      <c r="B4" s="4"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="10" t="s">
         <v>15</v>
       </c>
     </row>
@@ -776,15 +799,15 @@
       <c r="B4" s="2"/>
     </row>
     <row r="5" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="3">
+      <c r="A5" s="12">
         <f ca="1">NOW()</f>
-        <v>46187.942677662038</v>
-      </c>
-      <c r="B5" s="3"/>
+        <v>46190.540767939812</v>
+      </c>
+      <c r="B5" s="12"/>
     </row>
     <row r="6" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7"/>
+      <c r="A6" s="6"/>
+      <c r="B6" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -806,7 +829,7 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:1" ht="56.25" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Website update 2026-06-18 12:21:23
</commit_message>
<xml_diff>
--- a/build/source/lasvillasweb.xlsx
+++ b/build/source/lasvillasweb.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\lasvillasdebayamon\web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76E0939A-3A24-4F5C-8628-743F62F18C2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D85FF01-1933-46A5-8EE9-150CBF5A590D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -110,7 +110,7 @@
 de Puerto Rico</t>
   </si>
   <si>
-    <t>Como cada semana, también hoy tendremos la reunión informal de los miércoles en el gazebo a las 7:00 p. m. Todos son bienvenidos para conversar y discutir temas relacionados con el condominio.</t>
+    <t>Cada miércoles a las 7:00 p. m. se celebra una reunión informal de residentes en el gazebo. Es una oportunidad para conversar sobre asuntos de interés para la comunidad. Todos los residentes son bienvenidos.</t>
   </si>
 </sst>
 </file>
@@ -228,11 +228,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -625,7 +625,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:1" ht="112.5" x14ac:dyDescent="0.3">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="12" t="s">
         <v>18</v>
       </c>
     </row>
@@ -799,11 +799,11 @@
       <c r="B4" s="2"/>
     </row>
     <row r="5" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="12">
+      <c r="A5" s="13">
         <f ca="1">NOW()</f>
-        <v>46190.540767939812</v>
-      </c>
-      <c r="B5" s="12"/>
+        <v>46191.512985879628</v>
+      </c>
+      <c r="B5" s="13"/>
     </row>
     <row r="6" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="6"/>

</xml_diff>

<commit_message>
Website update 2026-06-19 01:02:56
</commit_message>
<xml_diff>
--- a/build/source/lasvillasweb.xlsx
+++ b/build/source/lasvillasweb.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\lasvillasdebayamon\web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B2CB268-73F3-4E29-B355-9E52CCADEAF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{875215E9-B11A-4B06-B707-FCC8D95AD21E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Homepage" sheetId="1" r:id="rId1"/>
     <sheet name="Documentos" sheetId="2" r:id="rId2"/>
     <sheet name="Números útiles" sheetId="7" r:id="rId3"/>
     <sheet name="Enlaces útiles" sheetId="8" r:id="rId4"/>
-    <sheet name="Test 2" sheetId="9" r:id="rId5"/>
+    <sheet name="Test 556" sheetId="9" r:id="rId5"/>
     <sheet name="#header" sheetId="5" r:id="rId6"/>
     <sheet name="#footer" sheetId="6" r:id="rId7"/>
   </sheets>
@@ -785,7 +785,7 @@
     <row r="5" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <f ca="1">NOW()</f>
-        <v>46192.023207175924</v>
+        <v>46192.043317476855</v>
       </c>
       <c r="B5" s="12"/>
     </row>

</xml_diff>

<commit_message>
Website update 2026-06-19 02:14:07
</commit_message>
<xml_diff>
--- a/build/source/lasvillasweb.xlsx
+++ b/build/source/lasvillasweb.xlsx
@@ -1,25 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="Questa_cartella_di_lavoro"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\lasvillasdebayamon\web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{875215E9-B11A-4B06-B707-FCC8D95AD21E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24C14587-1B52-4DA0-B580-7F98C29824E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Homepage" sheetId="1" r:id="rId1"/>
     <sheet name="Documentos" sheetId="2" r:id="rId2"/>
-    <sheet name="Números útiles" sheetId="7" r:id="rId3"/>
-    <sheet name="Enlaces útiles" sheetId="8" r:id="rId4"/>
-    <sheet name="Test 556" sheetId="9" r:id="rId5"/>
-    <sheet name="#header" sheetId="5" r:id="rId6"/>
-    <sheet name="#footer" sheetId="6" r:id="rId7"/>
+    <sheet name="Números útiles" sheetId="3" r:id="rId3"/>
+    <sheet name="Enlaces útiles" sheetId="4" r:id="rId4"/>
+    <sheet name="#header" sheetId="5" r:id="rId5"/>
+    <sheet name="#footer" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="Desc">'#header'!$A$4</definedName>
@@ -27,9 +26,6 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -37,6 +33,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -44,76 +42,174 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+  <si>
+    <t>Números útiles</t>
+  </si>
+  <si>
+    <t>Bomberos:</t>
+  </si>
+  <si>
+    <t>Emergencias generales:</t>
+  </si>
+  <si>
+    <t>911</t>
+  </si>
+  <si>
+    <t>Manejo de Emergencias Bayamón (AMMEAD):</t>
+  </si>
+  <si>
+    <t>Sala de Emergencias Bayamón Medical Center:</t>
+  </si>
+  <si>
+    <t>Reglamento del condominio vigente</t>
+  </si>
+  <si>
+    <t>Enlaces útiles</t>
+  </si>
+  <si>
+    <t>Busqueda de Estatus de FHA en Condominios</t>
+  </si>
   <si>
     <t>Ultima actualizacion:</t>
   </si>
   <si>
-    <t>Regolamento de condominio vigente:</t>
-  </si>
-  <si>
-    <t>pdf download</t>
-  </si>
-  <si>
-    <t>Documentos utiles</t>
-  </si>
-  <si>
-    <t>A raíz del éxito de la comunidad de WhatsApp, este espacio estará dedicado a la publicación de los principales temas e iniciativas del condominio.
-Este sitio no es una publicación oficial de la administración del condominio, sino una iniciativa privada compartida con toda la comunidad.
+    <t>Las Villas de Bayamon</t>
+  </si>
+  <si>
+    <t>Proyecto Informativo Gratuito</t>
+  </si>
+  <si>
+    <t>Caseta de Seguridad:</t>
+  </si>
+  <si>
+    <t>(787) 946-4623</t>
+  </si>
+  <si>
+    <t>(787) 946-7219</t>
+  </si>
+  <si>
+    <t>(787) 230-7074</t>
+  </si>
+  <si>
+    <t>(787) 785-3030</t>
+  </si>
+  <si>
+    <t>(787) 785-9620</t>
+  </si>
+  <si>
+    <t>(787) 786-6400</t>
+  </si>
+  <si>
+    <t>(787) 620-8181</t>
+  </si>
+  <si>
+    <t>Unique Security</t>
+  </si>
+  <si>
+    <t>(787) 689-3844</t>
+  </si>
+  <si>
+    <t>Administración Oficial:</t>
+  </si>
+  <si>
+    <t>Policía:</t>
+  </si>
+  <si>
+    <t>DACO
+Departamento de Asuntos del Consumidor de Puerto Rico</t>
+  </si>
+  <si>
+    <t>Documentos útiles</t>
+  </si>
+  <si>
+    <t>Grupo de WhatsApp</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">A raíz del éxito de la comunidad de WhatsApp, este espacio estará dedicado a la publicación de los principales temas e iniciativas del nuestra comunidad.
+Este sitio </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>no</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>es</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> una publicación </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>oficial</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> de la administración del condominio, sino una iniciativa privada compartida con toda la comunidad.
 Este es un servicio gratuito,
 y próximamente se publicarán los contactos para mejorar la comunicación entre los residentes.</t>
-  </si>
-  <si>
-    <t>Números útiles</t>
-  </si>
-  <si>
-    <t>Servicio de vigilancia:</t>
-  </si>
-  <si>
-    <t>787 230-7074</t>
-  </si>
-  <si>
-    <t>787 946-4623</t>
-  </si>
-  <si>
-    <t>Agente Administrador:</t>
-  </si>
-  <si>
-    <t>785 785-3030</t>
-  </si>
-  <si>
-    <t>Bomberos:</t>
-  </si>
-  <si>
-    <t>Policia:</t>
-  </si>
-  <si>
-    <t>787 785-9620</t>
-  </si>
-  <si>
-    <t>Enlaces útiles</t>
-  </si>
-  <si>
-    <t>https://www.daco.pr.gov/</t>
-  </si>
-  <si>
-    <t>Las Villas de Bayamon
-projecto informativo gratuito
-2026</t>
-  </si>
-  <si>
-    <t>DACO
-Departamento de Asuntos
-del Consumidor
-de Puerto Rico</t>
+    </r>
+  </si>
+  <si>
+    <t>Enviar sugerencias y/o comentarios al siguiente email:</t>
+  </si>
+  <si>
+    <t>lasvillasdebayamon@zohomail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$-540A]dddd\,\ mmmm\ d\,\ yyyy\ /\ hh\.mm"/>
+    <numFmt numFmtId="165" formatCode="[$-540A]dddd\,\ mmmm\ d\,\ yyyy\ \ \ \ h:mm\ AM/PM"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -155,7 +251,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
+      <sz val="14"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -180,17 +276,11 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -200,19 +290,55 @@
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -252,7 +378,7 @@
         <xdr:cNvPr id="5" name="Immagine 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DD27D30D-BA65-4EDC-962B-CF2CAD85C44B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -274,6 +400,9 @@
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -291,17 +420,17 @@
       <xdr:rowOff>47626</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>495300</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>3213270</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>72432</xdr:rowOff>
+      <xdr:rowOff>28575</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Immagine 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0CBE88B0-1FAA-4670-BA19-F643DCD78102}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -318,11 +447,14 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="28576" y="1333501"/>
-          <a:ext cx="3267074" cy="1739306"/>
+          <a:ext cx="3184694" cy="1695449"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -595,18 +727,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Foglio1"/>
   <dimension ref="A2"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="45.85546875" style="4" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" style="4" customWidth="1"/>
-    <col min="3" max="3" width="19.5703125" style="4" customWidth="1"/>
-    <col min="4" max="4" width="28.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="4"/>
+    <col min="1" max="1" width="45.85546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="28.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" style="2" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:1" ht="281.25" x14ac:dyDescent="0.3">
-      <c r="A2" s="11" t="s">
-        <v>4</v>
+    <row r="2" spans="1:1" ht="281.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -617,32 +748,31 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13BC1153-3F6C-40E1-89DB-D14060C3AC9B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Foglio2"/>
   <dimension ref="A2:A5"/>
-  <sheetFormatPr defaultColWidth="39.5703125" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="39.42578125" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16384" width="39.5703125" style="4"/>
+    <col min="1" max="1" width="45.85546875" style="2" customWidth="1"/>
+    <col min="2" max="16384" width="39.42578125" style="2"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
-        <v>1</v>
+      <c r="A4" s="3" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
-        <v>2</v>
-      </c>
+      <c r="A5" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A5" r:id="rId1" xr:uid="{07D0A0B5-0109-4276-9387-CD68095ACA66}"/>
+    <hyperlink ref="A4" r:id="rId1" display="Reglamento de condominio vigente:" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -650,174 +780,238 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36F7898C-6129-4D6F-BF35-20B4A0C8CE7F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Foglio3"/>
-  <dimension ref="A2:A14"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:A27"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.42578125" style="4" customWidth="1"/>
-    <col min="2" max="2" width="16.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="4"/>
+    <col min="1" max="1" width="45.85546875" style="8" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" style="2" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>5</v>
+      <c r="A2" s="7" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
-        <v>9</v>
+      <c r="A4" s="8" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
-        <v>8</v>
+      <c r="A5" s="9" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" s="8"/>
+      <c r="A6" s="9"/>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
-        <v>6</v>
+      <c r="A7" s="12" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8" s="8" t="s">
-        <v>7</v>
+      <c r="A8" s="9" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A9" s="8"/>
+      <c r="A9" s="9"/>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
-        <v>11</v>
+      <c r="A10" s="12" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A11" s="8" t="s">
-        <v>10</v>
+      <c r="A11" s="9" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A12" s="8"/>
+      <c r="A12" s="9" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
-        <v>12</v>
-      </c>
+      <c r="A13" s="9"/>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
-        <v>13</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A15" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A16" s="9"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" s="10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" s="11" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" ht="37.5" x14ac:dyDescent="0.3">
+      <c r="A23" s="10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A24" s="11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" ht="37.5" x14ac:dyDescent="0.3">
+      <c r="A26" s="10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A27" s="11" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36B8FD88-522D-4664-8FE8-C1F0587B8124}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Foglio4"/>
-  <dimension ref="A2:B5"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:B8"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="4"/>
+    <col min="1" max="1" width="45.85546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" style="2" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="75" x14ac:dyDescent="0.3">
-      <c r="A4" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="5"/>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="10" t="s">
-        <v>15</v>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="56.25" x14ac:dyDescent="0.3">
+      <c r="A4" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="3"/>
+    </row>
+    <row r="6" spans="1:2" ht="37.5" x14ac:dyDescent="0.3">
+      <c r="A6" s="14" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="15" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A5" r:id="rId1" xr:uid="{CFB0E60D-4B48-4A60-870C-5DDFBEEE89AE}"/>
+    <hyperlink ref="A4" r:id="rId1" display="DACO_x000a_Departamento de Asuntos_x000a_del Consumidor_x000a_de Puerto Rico" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
+    <hyperlink ref="A6" r:id="rId2" xr:uid="{00000000-0004-0000-0300-000001000000}"/>
+    <hyperlink ref="A8" r:id="rId3" xr:uid="{043A8B67-D743-40E4-9603-A5F6634A1F01}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId4"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D480487E-9BB2-412D-B903-C394CFDD7469}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EC846B1-29CA-4378-91FD-BEA3AC8F6F48}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr codeName="Foglio5"/>
-  <dimension ref="A4:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A4:A6"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="45.85546875" style="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="2"/>
-    </row>
-    <row r="5" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="12">
+    <row r="4" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="20">
         <f ca="1">NOW()</f>
-        <v>46192.043317476855</v>
-      </c>
-      <c r="B5" s="12"/>
-    </row>
-    <row r="6" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
+        <v>46192.091184259261</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="18"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A5:B5"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87CF910D-75B6-4C6D-9502-D7BB38A72D1D}">
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr codeName="Foglio6"/>
-  <dimension ref="A3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A3:A8"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="59.28515625" customWidth="1"/>
+    <col min="1" max="1" width="45.28515625" style="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:1" ht="56.25" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
-        <v>16</v>
+    <row r="3" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="37.5" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A8" s="21" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A8" r:id="rId1" xr:uid="{12C6D2D5-372C-4DF7-8E01-F2ACCFE70E7C}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Website update 2026-06-19 02:29:34
</commit_message>
<xml_diff>
--- a/build/source/lasvillasweb.xlsx
+++ b/build/source/lasvillasweb.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\lasvillasdebayamon\web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24C14587-1B52-4DA0-B580-7F98C29824E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A118440-1D7C-412F-AD3B-8DDAE9D335E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Homepage" sheetId="1" r:id="rId1"/>
@@ -278,7 +278,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -310,15 +310,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -339,6 +330,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -905,30 +908,30 @@
   <dimension ref="A2:B8"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="45.85546875" style="2" customWidth="1"/>
+    <col min="1" max="1" width="45.85546875" style="22" customWidth="1"/>
     <col min="2" max="2" width="16.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.140625" style="2" customWidth="1"/>
     <col min="4" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="20" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="56.25" x14ac:dyDescent="0.3">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="23" t="s">
         <v>24</v>
       </c>
       <c r="B4" s="3"/>
     </row>
-    <row r="6" spans="1:2" ht="37.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="14" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="21" t="s">
         <v>26</v>
       </c>
     </row>
@@ -949,22 +952,22 @@
   <dimension ref="A4:A6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="45.85546875" style="19" customWidth="1"/>
+    <col min="1" max="1" width="45.85546875" style="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="4" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="14" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="20">
+      <c r="A5" s="17">
         <f ca="1">NOW()</f>
-        <v>46192.091184259261</v>
+        <v>46192.098760763889</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="18"/>
+      <c r="A6" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -979,11 +982,11 @@
   <dimension ref="A3:A8"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="45.28515625" style="22" customWidth="1"/>
+    <col min="1" max="1" width="45.28515625" style="19" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="13" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1003,7 +1006,7 @@
       </c>
     </row>
     <row r="8" spans="1:1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="18" t="s">
         <v>29</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Website update 2026-06-20 16:44:20
</commit_message>
<xml_diff>
--- a/build/source/lasvillasweb.xlsx
+++ b/build/source/lasvillasweb.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr codeName="Questa_cartella_di_lavoro"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\lasvillasdebayamon\web\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\lasvillasdebayamon\web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A118440-1D7C-412F-AD3B-8DDAE9D335E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D85FF01-1933-46A5-8EE9-150CBF5A590D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Homepage" sheetId="1" r:id="rId1"/>
     <sheet name="Documentos" sheetId="2" r:id="rId2"/>
-    <sheet name="Números útiles" sheetId="3" r:id="rId3"/>
-    <sheet name="Enlaces útiles" sheetId="4" r:id="rId4"/>
+    <sheet name="Números útiles" sheetId="7" r:id="rId3"/>
+    <sheet name="Enlaces útiles" sheetId="8" r:id="rId4"/>
     <sheet name="#header" sheetId="5" r:id="rId5"/>
     <sheet name="#footer" sheetId="6" r:id="rId6"/>
   </sheets>
@@ -26,6 +26,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -33,185 +36,91 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
-  <si>
-    <t>Números útiles</t>
-  </si>
-  <si>
-    <t>Bomberos:</t>
-  </si>
-  <si>
-    <t>Emergencias generales:</t>
-  </si>
-  <si>
-    <t>911</t>
-  </si>
-  <si>
-    <t>Manejo de Emergencias Bayamón (AMMEAD):</t>
-  </si>
-  <si>
-    <t>Sala de Emergencias Bayamón Medical Center:</t>
-  </si>
-  <si>
-    <t>Reglamento del condominio vigente</t>
-  </si>
-  <si>
-    <t>Enlaces útiles</t>
-  </si>
-  <si>
-    <t>Busqueda de Estatus de FHA en Condominios</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Ultima actualizacion:</t>
   </si>
   <si>
-    <t>Las Villas de Bayamon</t>
-  </si>
-  <si>
-    <t>Proyecto Informativo Gratuito</t>
-  </si>
-  <si>
-    <t>Caseta de Seguridad:</t>
-  </si>
-  <si>
-    <t>(787) 946-4623</t>
-  </si>
-  <si>
-    <t>(787) 946-7219</t>
-  </si>
-  <si>
-    <t>(787) 230-7074</t>
-  </si>
-  <si>
-    <t>(787) 785-3030</t>
-  </si>
-  <si>
-    <t>(787) 785-9620</t>
-  </si>
-  <si>
-    <t>(787) 786-6400</t>
-  </si>
-  <si>
-    <t>(787) 620-8181</t>
-  </si>
-  <si>
-    <t>Unique Security</t>
-  </si>
-  <si>
-    <t>(787) 689-3844</t>
-  </si>
-  <si>
-    <t>Administración Oficial:</t>
-  </si>
-  <si>
-    <t>Policía:</t>
-  </si>
-  <si>
-    <t>DACO
-Departamento de Asuntos del Consumidor de Puerto Rico</t>
-  </si>
-  <si>
-    <t>Documentos útiles</t>
-  </si>
-  <si>
-    <t>Grupo de WhatsApp</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">A raíz del éxito de la comunidad de WhatsApp, este espacio estará dedicado a la publicación de los principales temas e iniciativas del nuestra comunidad.
-Este sitio </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>no</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>es</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> una publicación </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>oficial</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> de la administración del condominio, sino una iniciativa privada compartida con toda la comunidad.
+    <t>Regolamento de condominio vigente:</t>
+  </si>
+  <si>
+    <t>pdf download</t>
+  </si>
+  <si>
+    <t>Documentos utiles</t>
+  </si>
+  <si>
+    <t>A raíz del éxito de la comunidad de WhatsApp, este espacio estará dedicado a la publicación de los principales temas e iniciativas del condominio.
+Este sitio no es una publicación oficial de la administración del condominio, sino una iniciativa privada compartida con toda la comunidad.
 Este es un servicio gratuito,
 y próximamente se publicarán los contactos para mejorar la comunicación entre los residentes.</t>
-    </r>
-  </si>
-  <si>
-    <t>Enviar sugerencias y/o comentarios al siguiente email:</t>
-  </si>
-  <si>
-    <t>lasvillasdebayamon@zohomail.com</t>
+  </si>
+  <si>
+    <t>Números útiles</t>
+  </si>
+  <si>
+    <t>Servicio de vigilancia:</t>
+  </si>
+  <si>
+    <t>787 230-7074</t>
+  </si>
+  <si>
+    <t>787 946-4623</t>
+  </si>
+  <si>
+    <t>Agente Administrador:</t>
+  </si>
+  <si>
+    <t>785 785-3030</t>
+  </si>
+  <si>
+    <t>Bomberos:</t>
+  </si>
+  <si>
+    <t>Policia:</t>
+  </si>
+  <si>
+    <t>787 785-9620</t>
+  </si>
+  <si>
+    <t>Enlaces útiles</t>
+  </si>
+  <si>
+    <t>https://www.daco.pr.gov/</t>
+  </si>
+  <si>
+    <t>Las Villas de Bayamon
+projecto informativo gratuito
+2026</t>
+  </si>
+  <si>
+    <t>DACO
+Departamento de Asuntos
+del Consumidor
+de Puerto Rico</t>
+  </si>
+  <si>
+    <t>Cada miércoles a las 7:00 p. m. se celebra una reunión informal de residentes en el gazebo. Es una oportunidad para conversar sobre asuntos de interés para la comunidad. Todos los residentes son bienvenidos.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-540A]dddd\,\ mmmm\ d\,\ yyyy\ /\ hh\.mm"/>
-    <numFmt numFmtId="165" formatCode="[$-540A]dddd\,\ mmmm\ d\,\ yyyy\ \ \ \ h:mm\ AM/PM"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -251,18 +160,30 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="14"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -276,77 +197,47 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
+    <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -367,13 +258,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>57151</xdr:colOff>
-      <xdr:row>2</xdr:row>
+      <xdr:row>4</xdr:row>
       <xdr:rowOff>9524</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
       <xdr:colOff>3132395</xdr:colOff>
-      <xdr:row>14</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>95785</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -381,7 +272,7 @@
         <xdr:cNvPr id="5" name="Immagine 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DD27D30D-BA65-4EDC-962B-CF2CAD85C44B}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -403,9 +294,6 @@
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -423,17 +311,17 @@
       <xdr:rowOff>47626</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>3213270</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>495300</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:rowOff>72432</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Immagine 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0CBE88B0-1FAA-4670-BA19-F643DCD78102}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -450,14 +338,11 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="28576" y="1333501"/>
-          <a:ext cx="3184694" cy="1695449"/>
+          <a:ext cx="3267074" cy="1739306"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -729,18 +614,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Foglio1"/>
-  <dimension ref="A2"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:A4"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="45.85546875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="28.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="2" customWidth="1"/>
-    <col min="4" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="45.85546875" style="3" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="19.5703125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="28.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:1" ht="281.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
-        <v>27</v>
+    <row r="2" spans="1:1" ht="112.5" x14ac:dyDescent="0.3">
+      <c r="A2" s="12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="281.25" x14ac:dyDescent="0.3">
+      <c r="A4" s="11" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -751,31 +642,32 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13BC1153-3F6C-40E1-89DB-D14060C3AC9B}">
   <sheetPr codeName="Foglio2"/>
   <dimension ref="A2:A5"/>
-  <sheetFormatPr defaultColWidth="39.42578125" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="39.5703125" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="45.85546875" style="2" customWidth="1"/>
-    <col min="2" max="16384" width="39.42578125" style="2"/>
+    <col min="1" max="16384" width="39.5703125" style="3"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>25</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" s="5"/>
+      <c r="A5" s="7" t="s">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A4" r:id="rId1" display="Reglamento de condominio vigente:" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="A5" r:id="rId1" xr:uid="{07D0A0B5-0109-4276-9387-CD68095ACA66}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -783,193 +675,144 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36F7898C-6129-4D6F-BF35-20B4A0C8CE7F}">
   <sheetPr codeName="Foglio3"/>
-  <dimension ref="A2:A27"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:A14"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="45.85546875" style="8" customWidth="1"/>
-    <col min="2" max="2" width="16.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="2" customWidth="1"/>
-    <col min="4" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="30.42578125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
-        <v>0</v>
+      <c r="A2" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="8" t="s">
-        <v>22</v>
+      <c r="A4" s="3" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
-        <v>13</v>
+      <c r="A5" s="8" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" s="9"/>
+      <c r="A6" s="8"/>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" s="8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" s="8"/>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A12" s="8"/>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A9" s="9"/>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A10" s="12" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A11" s="9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A12" s="9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A13" s="9"/>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A15" s="9" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A16" s="9"/>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" s="8" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" s="9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A20" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A21" s="11" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" ht="37.5" x14ac:dyDescent="0.3">
-      <c r="A23" s="10" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A24" s="11" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" ht="37.5" x14ac:dyDescent="0.3">
-      <c r="A26" s="10" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A27" s="11" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36B8FD88-522D-4664-8FE8-C1F0587B8124}">
   <sheetPr codeName="Foglio4"/>
-  <dimension ref="A2:B8"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:B5"/>
+  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="45.85546875" style="22" customWidth="1"/>
-    <col min="2" max="2" width="16.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="2" customWidth="1"/>
-    <col min="4" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="30.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="20" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="56.25" x14ac:dyDescent="0.3">
-      <c r="A4" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="B4" s="3"/>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="21" t="s">
-        <v>26</v>
+      <c r="A2" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="75" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="4"/>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="10" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A4" r:id="rId1" display="DACO_x000a_Departamento de Asuntos_x000a_del Consumidor_x000a_de Puerto Rico" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
-    <hyperlink ref="A6" r:id="rId2" xr:uid="{00000000-0004-0000-0300-000001000000}"/>
-    <hyperlink ref="A8" r:id="rId3" xr:uid="{043A8B67-D743-40E4-9603-A5F6634A1F01}"/>
+    <hyperlink ref="A5" r:id="rId1" xr:uid="{CFB0E60D-4B48-4A60-870C-5DDFBEEE89AE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EC846B1-29CA-4378-91FD-BEA3AC8F6F48}">
   <sheetPr codeName="Foglio5"/>
-  <dimension ref="A4:A6"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A4:B6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="45.85546875" style="16" customWidth="1"/>
+    <col min="1" max="1" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="17">
+    <row r="4" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="2"/>
+    </row>
+    <row r="5" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A5" s="13">
         <f ca="1">NOW()</f>
-        <v>46192.098760763889</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="15"/>
+        <v>46191.512985879628</v>
+      </c>
+      <c r="B5" s="13"/>
+    </row>
+    <row r="6" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A6" s="6"/>
+      <c r="B6" s="6"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A5:B5"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -977,44 +820,20 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87CF910D-75B6-4C6D-9502-D7BB38A72D1D}">
   <sheetPr codeName="Foglio6"/>
-  <dimension ref="A3:A8"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="45.28515625" style="19" customWidth="1"/>
+    <col min="1" max="1" width="59.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" ht="37.5" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A8" s="18" t="s">
-        <v>29</v>
+    <row r="3" spans="1:1" ht="56.25" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A8" r:id="rId1" xr:uid="{12C6D2D5-372C-4DF7-8E01-F2ACCFE70E7C}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Website update 2026-06-20 17:24:21
</commit_message>
<xml_diff>
--- a/build/source/lasvillasweb.xlsx
+++ b/build/source/lasvillasweb.xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\lasvillasdebayamon\web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D85FF01-1933-46A5-8EE9-150CBF5A590D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F965EE9B-7228-4630-8B70-E5EAC5BDE8DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Homepage" sheetId="1" r:id="rId1"/>
-    <sheet name="Documentos" sheetId="2" r:id="rId2"/>
-    <sheet name="Números útiles" sheetId="7" r:id="rId3"/>
-    <sheet name="Enlaces útiles" sheetId="8" r:id="rId4"/>
-    <sheet name="#header" sheetId="5" r:id="rId5"/>
-    <sheet name="#footer" sheetId="6" r:id="rId6"/>
+    <sheet name="Anuncios" sheetId="9" r:id="rId2"/>
+    <sheet name="Documentos" sheetId="2" r:id="rId3"/>
+    <sheet name="Números útiles" sheetId="7" r:id="rId4"/>
+    <sheet name="Enlaces útiles" sheetId="8" r:id="rId5"/>
+    <sheet name="#header" sheetId="5" r:id="rId6"/>
+    <sheet name="#footer" sheetId="6" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="Desc">'#header'!$A$4</definedName>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Ultima actualizacion:</t>
   </si>
@@ -111,6 +112,9 @@
   </si>
   <si>
     <t>Cada miércoles a las 7:00 p. m. se celebra una reunión informal de residentes en el gazebo. Es una oportunidad para conversar sobre asuntos de interés para la comunidad. Todos los residentes son bienvenidos.</t>
+  </si>
+  <si>
+    <t>anu</t>
   </si>
 </sst>
 </file>
@@ -642,6 +646,21 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A94208C-A5E1-410D-86D3-F1B3F1798E0F}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13BC1153-3F6C-40E1-89DB-D14060C3AC9B}">
   <sheetPr codeName="Foglio2"/>
   <dimension ref="A2:A5"/>
@@ -674,7 +693,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36F7898C-6129-4D6F-BF35-20B4A0C8CE7F}">
   <sheetPr codeName="Foglio3"/>
   <dimension ref="A2:A14"/>
@@ -746,7 +765,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36B8FD88-522D-4664-8FE8-C1F0587B8124}">
   <sheetPr codeName="Foglio4"/>
   <dimension ref="A2:B5"/>
@@ -782,7 +801,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EC846B1-29CA-4378-91FD-BEA3AC8F6F48}">
   <sheetPr codeName="Foglio5"/>
   <dimension ref="A4:B6"/>
@@ -801,7 +820,7 @@
     <row r="5" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="13">
         <f ca="1">NOW()</f>
-        <v>46191.512985879628</v>
+        <v>46193.724751620372</v>
       </c>
       <c r="B5" s="13"/>
     </row>
@@ -819,7 +838,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87CF910D-75B6-4C6D-9502-D7BB38A72D1D}">
   <sheetPr codeName="Foglio6"/>
   <dimension ref="A3"/>

</xml_diff>